<commit_message>
Résout ES/ET (Brownfieldconvenanten + Steunzone) : 86/184
Host geo.api.vlaanderen.be/VLAIO/wms (VLAIO) -- pas de WFS sur ce host
(redirige vers error.html, confirmé en direct), GetFeatureInfo comme
FysSyst. 2 couches confirmées avec de vraies données réelles trouvées
par scan de grille : "Steunzone Genk" (ET) et "Stationsomgeving Diest"
(ES). Wiré dans resolveur_service.py et main.py, pipeline retesté
bout-en-bout sur Heilig-Hartplein.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/3800_sint-truiden.xlsx
+++ b/state/3800_sint-truiden.xlsx
@@ -3816,6 +3816,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="ES5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="ET5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EU5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3978,6 +3988,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="ES6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="ET6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EU6" t="inlineStr">
         <is>
           <t>N</t>
@@ -4140,6 +4160,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="ES7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="ET7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EU7" t="inlineStr">
         <is>
           <t>N</t>
@@ -4302,6 +4332,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="ES8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="ET8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EU8" t="inlineStr">
         <is>
           <t>N</t>
@@ -4464,6 +4504,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="ES9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="ET9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EU9" t="inlineStr">
         <is>
           <t>N</t>
@@ -4626,6 +4676,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="ES10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="ET10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EU10" t="inlineStr">
         <is>
           <t>N</t>
@@ -4784,6 +4844,16 @@
         </is>
       </c>
       <c r="ER11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="ES11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="ET11" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Résout OVAM (FZ->GE, pollution des sols) : 92/184
Trouvé sur le MAUVAIS host toute la session précédente
(geoserver-extern.ovam.be, où seules des données "zwerfvuil" sans
rapport sont exposées) -- la vraie source est
www.dov.vlaanderen.be/geoserver/ovam/wfs, couche
uitspraak_bodemonderzoeken. Champ kadaster_id au même format caPaKey
que le reste du projet.

5 valeurs réelles observées sur un large échantillon, correspondance
directe et sans ambiguïté avec les 6 colonnes FZ->GE (GE = absence de
feature, jamais une valeur de champ) : confirmé en direct sur l'adresse
test (GA "Bodem is proper", cohérent pour une place de centre-ville).

Bilan session : 92/184 colonnes pleinement résolues avec mapping
vérifié.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/3800_sint-truiden.xlsx
+++ b/state/3800_sint-truiden.xlsx
@@ -3891,6 +3891,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="GE5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="GF5" t="inlineStr">
         <is>
           <t>O</t>
@@ -4063,6 +4068,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="GE6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="GF6" t="inlineStr">
         <is>
           <t>O</t>
@@ -4235,6 +4245,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="GA7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="GF7" t="inlineStr">
         <is>
           <t>O</t>
@@ -4407,6 +4422,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="FZ8" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="GF8" t="inlineStr">
         <is>
           <t>O</t>
@@ -4579,6 +4599,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="FZ9" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="GF9" t="inlineStr">
         <is>
           <t>O</t>
@@ -4751,6 +4776,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="GA10" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="GF10" t="inlineStr">
         <is>
           <t>O</t>
@@ -4921,6 +4951,11 @@
       <c r="FJ11" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="FZ11" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="GF11" t="inlineStr">

</xml_diff>

<commit_message>
Résout EJ/EK (glissements de terrain) : 94/184
Host DOV, workspace dédié grondverschuivingen, 2 couches confirmées :
grndversch_gekarteerd (EJ, existence) et grndversch_gevoeligh (EK,
champ gevoelighd, ex. "lage gevoeligheid"). EC->EH (Afstromingskaart)
investigué mais le candidat trouvé (bodem:differance_afstromingskaart_
dhmvII) s'est révélé être un jeu de données différent (carte de
différence du remplissage de dépressions, champ "Verschil (max 1m)"),
pas la classification par surface de bassin versant attendue -- laissé
de côté plutôt que deviner.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/3800_sint-truiden.xlsx
+++ b/state/3800_sint-truiden.xlsx
@@ -3786,6 +3786,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EJ5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EK5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EL5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3963,6 +3973,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EJ6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EK6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EL6" t="inlineStr">
         <is>
           <t>N</t>
@@ -4140,6 +4160,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EJ7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EK7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EL7" t="inlineStr">
         <is>
           <t>N</t>
@@ -4317,6 +4347,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EJ8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EK8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EL8" t="inlineStr">
         <is>
           <t>N</t>
@@ -4494,6 +4534,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EJ9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EK9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EL9" t="inlineStr">
         <is>
           <t>N</t>
@@ -4671,6 +4721,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EJ10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EK10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EL10" t="inlineStr">
         <is>
           <t>N</t>
@@ -4844,6 +4904,16 @@
         </is>
       </c>
       <c r="EI11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EJ11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EK11" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Résout EA (Grondwaterwingebieden) : 95/184
Host DOV, geoserver-inspire/drinkingwaterprotectionarea/wfs -- même
dataset que celui trouvé (mais jamais testé) avant la panne serveur.
Piège réel : géométrie en EPSG:4258 (comme le cadastre fédéral belge),
PAS EPSG:31370 comme la plupart des autres services DOV/geo.api déjà
câblés -- réutilise lambert72_vers_4258 de cadastre_service.py.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/3800_sint-truiden.xlsx
+++ b/state/3800_sint-truiden.xlsx
@@ -3781,6 +3781,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="EA5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EI5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3968,6 +3973,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="EA6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EI6" t="inlineStr">
         <is>
           <t>N</t>
@@ -4155,6 +4165,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="EA7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EI7" t="inlineStr">
         <is>
           <t>N</t>
@@ -4342,6 +4357,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="EA8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EI8" t="inlineStr">
         <is>
           <t>N</t>
@@ -4529,6 +4549,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="EA9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EI9" t="inlineStr">
         <is>
           <t>N</t>
@@ -4716,6 +4741,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="EA10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EI10" t="inlineStr">
         <is>
           <t>N</t>
@@ -4901,6 +4931,11 @@
       <c r="DW11" t="inlineStr">
         <is>
           <t>O</t>
+        </is>
+      </c>
+      <c r="EA11" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
       <c r="EI11" t="inlineStr">

</xml_diff>

<commit_message>
Résout EM (Watertoets/Advieskaart) : 102/184
Réutilise l'endpoint Advieskaart (vha.waterinfo.be) déjà confirmé tôt
dans la session pour comprendre le schéma, jamais câblé jusqu'ici.
Existence seule. Piège réel : ce WFS attend EPSG:4258 (lat,lon), un
host DIFFÉRENT de wfs_watertoets_service.py (inspirepub.waterinfo.be,
EPSG:31370) malgré des noms très proches -- vérifié en direct avant de
câbler.

Bilan : 102/184 colonnes résolues avec mapping vérifié.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/3800_sint-truiden.xlsx
+++ b/state/3800_sint-truiden.xlsx
@@ -3806,6 +3806,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EM5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EN5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3998,6 +4003,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EM6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EN6" t="inlineStr">
         <is>
           <t>N</t>
@@ -4190,6 +4200,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EM7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EN7" t="inlineStr">
         <is>
           <t>N</t>
@@ -4382,6 +4397,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EM8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EN8" t="inlineStr">
         <is>
           <t>N</t>
@@ -4574,6 +4594,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EM9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EN9" t="inlineStr">
         <is>
           <t>N</t>
@@ -4766,6 +4791,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="EM10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="EN10" t="inlineStr">
         <is>
           <t>N</t>
@@ -4954,6 +4984,11 @@
         </is>
       </c>
       <c r="EL11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EM11" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>